<commit_message>
feat(fonts): preserve Excel font family and add global font override settings
</commit_message>
<xml_diff>
--- a/templates/CREDIT_NOTE.xlsx
+++ b/templates/CREDIT_NOTE.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Credit Note</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>{{note_ref}}</t>
+  </si>
+  <si>
+    <t>{{@qr 'testmeanyway' }}</t>
   </si>
 </sst>
 </file>
@@ -126,7 +129,7 @@
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +182,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -208,11 +219,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -275,15 +287,19 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -337,50 +353,6 @@
         <a:xfrm>
           <a:off x="0" y="154781"/>
           <a:ext cx="1034389" cy="1129639"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>257736</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>101691</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>571501</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>126625</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4919383" y="4796956"/>
-          <a:ext cx="1210236" cy="1974758"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -704,7 +676,7 @@
       </c>
       <c r="F6" s="19">
         <f ca="1">TODAY()</f>
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="G6" s="19"/>
     </row>
@@ -804,6 +776,10 @@
       <c r="D24" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="E24" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" s="26"/>
     </row>
     <row r="37" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
@@ -863,7 +839,7 @@
       <c r="G41" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="B20:C20"/>
@@ -876,14 +852,18 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E24:F24"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E24" r:id="rId1"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="89" orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="89" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddFooter>&amp;CNote: In case of any change please contact head office within 10 days of receipt of this Credit Note.
 Any claims after this time will not be accaptable.</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(colors): implement ExcelColorResolver for 100% fidelity on theme colors, tints, indexed, and direct RGB
</commit_message>
<xml_diff>
--- a/templates/CREDIT_NOTE.xlsx
+++ b/templates/CREDIT_NOTE.xlsx
@@ -15,7 +15,7 @@
     <sheet name="CREDIT_NOTE" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">CREDIT_NOTE!$A$2:$G$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">CREDIT_NOTE!$A$1:$G$38</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Credit Note</t>
   </si>
@@ -65,15 +65,6 @@
     <t>CNIC No. :</t>
   </si>
   <si>
-    <t>.1</t>
-  </si>
-  <si>
-    <t>.2</t>
-  </si>
-  <si>
-    <t>.3</t>
-  </si>
-  <si>
     <t>________________</t>
   </si>
   <si>
@@ -113,10 +104,16 @@
     <t>{{cnic}}</t>
   </si>
   <si>
-    <t>{{note_ref}}</t>
-  </si>
-  <si>
     <t>{{@qr 'testmeanyway' }}</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
   </si>
 </sst>
 </file>
@@ -129,7 +126,7 @@
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,13 +198,33 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -224,7 +241,7 @@
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -294,6 +311,14 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -313,55 +338,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>154781</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1034389</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>167334</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="154781"/>
-          <a:ext cx="1034389" cy="1129639"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -630,7 +606,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A3:G41"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" style="1" customWidth="1"/>
@@ -643,147 +619,180 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-    </row>
-    <row r="5" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A5" s="16" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+    </row>
+    <row r="3" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E6" s="3" t="s">
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F4" s="19">
         <f ca="1">TODAY()</f>
         <v>46318</v>
       </c>
-      <c r="G6" s="19"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E7" s="3" t="s">
+      <c r="G4" s="19"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="20">
+        <f ca="1">NOW()</f>
+        <v>46318.009781250003</v>
+      </c>
+      <c r="G5" s="20"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="G7" s="20"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="25"/>
       <c r="D10" s="25"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="25" t="s">
+      <c r="A11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="14" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="25" t="s">
+      <c r="B16" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="C16" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" s="14" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="E16" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="18"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8"/>
+    </row>
+    <row r="18" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="17">
+        <f>SUM(B16:B16)</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="17"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="F22" s="26"/>
+    </row>
+    <row r="35" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="10" t="s">
+    </row>
+    <row r="36" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" s="18"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="8"/>
-    </row>
-    <row r="20" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="17">
-        <f>SUM(B18:B18)</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="17"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D24" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E24" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="F24" s="26"/>
     </row>
     <row r="37" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B37" s="21"/>
       <c r="C37" s="21"/>
@@ -791,71 +800,45 @@
       <c r="E37" s="21"/>
       <c r="F37" s="21"/>
       <c r="G37" s="13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B38" s="21"/>
-      <c r="C38" s="21"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
-      <c r="G38" s="13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C40" s="11"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="13"/>
-    </row>
-    <row r="41" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="11"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="13"/>
+    </row>
+    <row r="39" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B11:D11"/>
     <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="E22:F22"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="E24" r:id="rId1"/>
+    <hyperlink ref="E22" r:id="rId1"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -864,6 +847,5 @@
     <oddFooter>&amp;CNote: In case of any change please contact head office within 10 days of receipt of this Credit Note.
 Any claims after this time will not be accaptable.</oddFooter>
   </headerFooter>
-  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(colors): implement ECMA-376 HLS luminance tinting for exact Excel color shades
</commit_message>
<xml_diff>
--- a/templates/CREDIT_NOTE.xlsx
+++ b/templates/CREDIT_NOTE.xlsx
@@ -199,16 +199,16 @@
       <family val="1"/>
     </font>
     <font>
+      <b/>
+      <u/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <u/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="0"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -222,7 +222,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.249977111117893"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -314,13 +314,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -662,7 +662,7 @@
       </c>
       <c r="F5" s="20">
         <f ca="1">NOW()</f>
-        <v>46318.009781250003</v>
+        <v>46318.010496990741</v>
       </c>
       <c r="G5" s="20"/>
     </row>
@@ -703,15 +703,15 @@
       <c r="A12" s="4"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">

</xml_diff>

<commit_message>
feat(engine): support Excel conditional formatting evaluation, loop expansion, and color scale heatmaps
</commit_message>
<xml_diff>
--- a/templates/CREDIT_NOTE.xlsx
+++ b/templates/CREDIT_NOTE.xlsx
@@ -15,7 +15,7 @@
     <sheet name="CREDIT_NOTE" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">CREDIT_NOTE!$A$1:$G$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">CREDIT_NOTE!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Credit Note</t>
   </si>
@@ -65,9 +65,6 @@
     <t>CNIC No. :</t>
   </si>
   <si>
-    <t>________________</t>
-  </si>
-  <si>
     <t>Approved By:</t>
   </si>
   <si>
@@ -104,9 +101,6 @@
     <t>{{cnic}}</t>
   </si>
   <si>
-    <t>{{@qr 'testmeanyway' }}</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -114,6 +108,9 @@
   </si>
   <si>
     <t>3</t>
+  </si>
+  <si>
+    <t>{{@qr dist_name + dist_city + subject width=80 height=80}}</t>
   </si>
 </sst>
 </file>
@@ -124,7 +121,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_-&quot;Rs&quot;* #,##0_-;\-&quot;Rs&quot;* #,##0_-;_-&quot;Rs&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -222,17 +219,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -241,93 +253,111 @@
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -606,243 +636,464 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.7109375" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="1.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="21" style="4" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="2.140625" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-    </row>
-    <row r="3" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+    </row>
+    <row r="2" spans="1:8" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="6"/>
+      <c r="B2" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+    </row>
+    <row r="3" spans="1:8" ht="20.25" x14ac:dyDescent="0.3">
+      <c r="A3" s="6"/>
+      <c r="B3" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E4" s="3" t="s">
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="19">
+      <c r="G4" s="29">
         <f ca="1">TODAY()</f>
         <v>46318</v>
       </c>
-      <c r="G4" s="19"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E5" s="3" t="s">
+      <c r="H4" s="29"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="30">
+        <f ca="1">NOW()</f>
+        <v>46318.069185185188</v>
+      </c>
+      <c r="H5" s="30"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+      <c r="B10" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="6"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="6"/>
+      <c r="B14" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="12"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+      <c r="B15" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="6"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="1:8" s="5" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="20">
-        <f ca="1">NOW()</f>
-        <v>46318.010496990741</v>
-      </c>
-      <c r="G5" s="20"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="27"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="14" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="10" t="s">
+      <c r="C17" s="18"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A18" s="6"/>
+      <c r="B18" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="28">
+        <f>SUM(C16:C16)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="28"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="34"/>
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="1:8" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="16"/>
+      <c r="B25" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="18"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="8"/>
-    </row>
-    <row r="18" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="17">
-        <f>SUM(B16:B16)</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="17"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" s="26" t="s">
+    </row>
+    <row r="26" spans="1:8" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="16"/>
+      <c r="B26" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F22" s="26"/>
-    </row>
-    <row r="35" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" s="21"/>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="13" t="s">
+    </row>
+    <row r="27" spans="1:8" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="16"/>
+      <c r="B27" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="19" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B36" s="21"/>
-      <c r="C36" s="21"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="B37" s="21"/>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
-      <c r="G37" s="13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C38" s="11"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="13"/>
-    </row>
-    <row r="39" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="22"/>
+    <row r="28" spans="1:8" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="16"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="19"/>
+    </row>
+    <row r="29" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" s="6"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="C8:E8"/>
   </mergeCells>
+  <conditionalFormatting sqref="C16">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <formula>250</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="E22" r:id="rId1"/>
+    <hyperlink ref="F22" r:id="rId1"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="89" orientation="portrait" r:id="rId2"/>
+  <pageSetup scale="91" fitToHeight="0" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddFooter>&amp;CNote: In case of any change please contact head office within 10 days of receipt of this Credit Note.
 Any claims after this time will not be accaptable.</oddFooter>

</xml_diff>

<commit_message>
chore(templates): update CREDIT_NOTE template
</commit_message>
<xml_diff>
--- a/templates/CREDIT_NOTE.xlsx
+++ b/templates/CREDIT_NOTE.xlsx
@@ -1083,11 +1083,6 @@
     <mergeCell ref="G16:H16"/>
     <mergeCell ref="C8:E8"/>
   </mergeCells>
-  <conditionalFormatting sqref="C16">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
-      <formula>250</formula>
-    </cfRule>
-  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="F22" r:id="rId1"/>
   </hyperlinks>

</xml_diff>